<commit_message>
Updated Bootloader, First Validation of Hardware
</commit_message>
<xml_diff>
--- a/Hardware/Controller/JLC_PCBA_BOM-DALI_EVG_Controller(V0.1).xlsx
+++ b/Hardware/Controller/JLC_PCBA_BOM-DALI_EVG_Controller(V0.1).xlsx
@@ -1,45 +1,167 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr codeName="ThisWorkbook"/>
+  <bookViews>
+    <workbookView tabRatio="600"/>
+  </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="JLC_PCBA_BOM-DALI_EVG_Controlle" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="JLC_PCBA_BOM-DALI_EVG_Controlle" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'JLC_PCBA_BOM-DALI_EVG_Controlle'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0"><![CDATA['JLC_PCBA_BOM-DALI_EVG_Controlle'!$1:$1]]></definedName>
   </definedNames>
-  <calcPr calcId="125725" calcMode="auto" fullCalcOnLoad="1" fullPrecision="1"/>
+  <calcPr calcId="125725" fullCalcOnLoad="1" fullPrecision="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="38">
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">JLCPCB Part #</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1525</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C13585</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C307331</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C59461</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C15849</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C19077450</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C19077439</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2488</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C8598</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5123971</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C720477</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C20917</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C15127</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C8326</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2145</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C25803</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C25271</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C11702</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C25741</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C102130</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C25744</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C21189</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C25092</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C22843</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C22859</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C22935</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C23162</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C25981</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C25810</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C4216</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C5299908</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C34731</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C6482</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
   <fonts count="5">
     <font>
+      <sz val="10"/>
       <name val="Tahoma"/>
       <charset val="0"/>
-      <sz val="10"/>
     </font>
     <font>
+      <sz val="10"/>
       <name val="Tahoma"/>
       <charset val="0"/>
-      <sz val="10"/>
     </font>
     <font>
+      <sz val="10"/>
       <name val="Tahoma"/>
       <charset val="0"/>
-      <sz val="10"/>
     </font>
     <font>
+      <sz val="10"/>
       <name val="Tahoma"/>
       <charset val="0"/>
-      <sz val="10"/>
     </font>
     <font>
+      <sz val="10"/>
       <name val="Tahoma"/>
       <charset val="0"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -225,37 +347,37 @@
     <xf numFmtId="9" fontId="4" fillId="2" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="31">
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="1" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="1" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" pivotButton="0" quotePrefix="1" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" pivotButton="0" quotePrefix="1" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" pivotButton="0" quotePrefix="1" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" pivotButton="0" quotePrefix="1" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" pivotButton="0" quotePrefix="1" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" pivotButton="0" quotePrefix="1" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" pivotButton="0" quotePrefix="1" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -265,7 +387,7 @@
     <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
     <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="" defaultPivotStyle=""/>
+  <tableStyles count="0"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -509,18 +631,21 @@
             </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:custDash/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:custDash/>
         </a:ln>
         <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:custDash/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -558,7 +683,7 @@
               <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
-          <a:sp3d>
+          <a:sp3d prstMaterial="warmMatte">
             <a:bevelT w="63500" h="25400"/>
           </a:sp3d>
         </a:effectStyle>
@@ -621,1161 +746,1451 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
-  <sheetFormatPr baseColWidth="0" defaultRowHeight="12.75"/>
+  <dimension ref="A1:G43"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col width="20.2109375" customWidth="1" style="30" min="1" max="2"/>
-    <col width="16.9609375" customWidth="1" style="30" min="3" max="3"/>
-    <col width="20.2109375" customWidth="1" style="30" min="4" max="6"/>
+    <col min="1" max="2" width="20.2109375" style="30" customWidth="1"/>
+    <col min="3" max="3" width="16.9609375" style="30" customWidth="1"/>
+    <col min="4" max="6" width="20.2109375" style="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="28" t="inlineStr">
-        <is>
-          <t>Comment</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">Comment</t>
         </is>
       </c>
       <c r="B1" s="29" t="inlineStr">
-        <is>
-          <t>Description</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">Description</t>
         </is>
       </c>
       <c r="C1" s="29" t="inlineStr">
-        <is>
-          <t>Value</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">Value</t>
         </is>
       </c>
       <c r="D1" s="29" t="inlineStr">
-        <is>
-          <t>Designator</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">Designator</t>
         </is>
       </c>
       <c r="E1" s="29" t="inlineStr">
-        <is>
-          <t>Footprint</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">Footprint</t>
         </is>
       </c>
       <c r="F1" s="29" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
+        <v/>
+        <is>
+          <t xml:space="preserve">Quantity</t>
+        </is>
+      </c>
+      <c r="G1" s="29" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="23" t="inlineStr">
-        <is>
-          <t>100nF</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">100nF</t>
         </is>
       </c>
       <c r="B2" s="18" t="inlineStr">
-        <is>
-          <t>Capacitor</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">Capacitor</t>
         </is>
       </c>
       <c r="C2" s="18" t="inlineStr">
-        <is>
-          <t>100nF, [NoParam]</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">100nF, [NoParam]</t>
         </is>
       </c>
       <c r="D2" s="18" t="inlineStr">
-        <is>
-          <t>C1, C3, C4, C11, C13, C14, C15</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">C1, C3, C4, C11, C13, C14, C15</t>
         </is>
       </c>
       <c r="E2" s="18" t="inlineStr">
-        <is>
-          <t>C0402</t>
-        </is>
-      </c>
-      <c r="F2" s="24" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">C0402</t>
+        </is>
+      </c>
+      <c r="F2" s="24">
         <v>7</v>
+      </c>
+      <c r="G2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="26" t="inlineStr">
-        <is>
-          <t>10uF/50V</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">10uF/50V</t>
         </is>
       </c>
       <c r="B3" s="19" t="inlineStr">
-        <is>
-          <t>Capacitor</t>
-        </is>
-      </c>
-      <c r="C3" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Capacitor</t>
+        </is>
+      </c>
+      <c r="C3" s="19"/>
       <c r="D3" s="19" t="inlineStr">
-        <is>
-          <t>C12, C19</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">C12, C19</t>
         </is>
       </c>
       <c r="E3" s="19" t="inlineStr">
-        <is>
-          <t>C1206</t>
-        </is>
-      </c>
-      <c r="F3" s="27" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">C1206</t>
+        </is>
+      </c>
+      <c r="F3" s="27">
         <v>2</v>
+      </c>
+      <c r="G3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="26" t="inlineStr">
-        <is>
-          <t>100nF/50V</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">100nF/50V</t>
         </is>
       </c>
       <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>Capacitor</t>
-        </is>
-      </c>
-      <c r="C4" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Capacitor</t>
+        </is>
+      </c>
+      <c r="C4" s="19"/>
       <c r="D4" s="19" t="inlineStr">
-        <is>
-          <t>C16</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">C16</t>
         </is>
       </c>
       <c r="E4" s="19" t="inlineStr">
-        <is>
-          <t>C0402</t>
-        </is>
-      </c>
-      <c r="F4" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">C0402</t>
+        </is>
+      </c>
+      <c r="F4" s="27">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>22uF</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">22uF</t>
         </is>
       </c>
       <c r="B5" s="19" t="inlineStr">
-        <is>
-          <t>Capacitor</t>
-        </is>
-      </c>
-      <c r="C5" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Capacitor</t>
+        </is>
+      </c>
+      <c r="C5" s="19"/>
       <c r="D5" s="19" t="inlineStr">
-        <is>
-          <t>C17, C18</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">C17, C18</t>
         </is>
       </c>
       <c r="E5" s="19" t="inlineStr">
-        <is>
-          <t>C0603</t>
-        </is>
-      </c>
-      <c r="F5" s="27" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">C0603</t>
+        </is>
+      </c>
+      <c r="F5" s="27">
         <v>2</v>
+      </c>
+      <c r="G5" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="26" t="inlineStr">
-        <is>
-          <t>1uF</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">1uF</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>Capacitor</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">Capacitor</t>
         </is>
       </c>
       <c r="C6" s="19" t="inlineStr">
-        <is>
-          <t>100nF</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">100nF</t>
         </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
-        <is>
-          <t>C21</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">C21</t>
         </is>
       </c>
       <c r="E6" s="19" t="inlineStr">
-        <is>
-          <t>C0603</t>
-        </is>
-      </c>
-      <c r="F6" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">C0603</t>
+        </is>
+      </c>
+      <c r="F6" s="27">
+        <v>1</v>
+      </c>
+      <c r="G6" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="26" t="inlineStr">
-        <is>
-          <t>220uF/50V</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">220uF/50V</t>
         </is>
       </c>
       <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>Polarized Capacitor (Axial)</t>
-        </is>
-      </c>
-      <c r="C7" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Polarized Capacitor (Axial)</t>
+        </is>
+      </c>
+      <c r="C7" s="19"/>
       <c r="D7" s="19" t="inlineStr">
-        <is>
-          <t>C24</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">C24</t>
         </is>
       </c>
       <c r="E7" s="19" t="inlineStr">
-        <is>
-          <t>CAPR-5mm</t>
-        </is>
-      </c>
-      <c r="F7" s="27" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">CAPR-5mm</t>
+        </is>
+      </c>
+      <c r="F7" s="27">
         <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="26" t="inlineStr">
-        <is>
-          <t>18V</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">18V</t>
         </is>
       </c>
       <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>Zener</t>
-        </is>
-      </c>
-      <c r="C8" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Zener</t>
+        </is>
+      </c>
+      <c r="C8" s="19"/>
       <c r="D8" s="19" t="inlineStr">
-        <is>
-          <t>D1</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">D1</t>
         </is>
       </c>
       <c r="E8" s="19" t="inlineStr">
-        <is>
-          <t>SOD-323</t>
-        </is>
-      </c>
-      <c r="F8" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">SOD-323</t>
+        </is>
+      </c>
+      <c r="F8" s="27">
+        <v>1</v>
+      </c>
+      <c r="G8" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="26" t="inlineStr">
-        <is>
-          <t>4.7V</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">4.7V</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>Zener</t>
-        </is>
-      </c>
-      <c r="C9" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Zener</t>
+        </is>
+      </c>
+      <c r="C9" s="19"/>
       <c r="D9" s="19" t="inlineStr">
-        <is>
-          <t>D2</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">D2</t>
         </is>
       </c>
       <c r="E9" s="19" t="inlineStr">
-        <is>
-          <t>SOD-323</t>
-        </is>
-      </c>
-      <c r="F9" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">SOD-323</t>
+        </is>
+      </c>
+      <c r="F9" s="27">
+        <v>1</v>
+      </c>
+      <c r="G9" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="26" t="inlineStr">
-        <is>
-          <t>MB10S</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">MB10S</t>
         </is>
       </c>
       <c r="B10" s="19" t="inlineStr"/>
-      <c r="C10" s="19" t="n"/>
+      <c r="C10" s="19"/>
       <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>D3</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">D3</t>
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
-        <is>
-          <t>SOIC245P670X290-4N</t>
-        </is>
-      </c>
-      <c r="F10" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">SOIC245P670X290-4N</t>
+        </is>
+      </c>
+      <c r="F10" s="27">
+        <v>1</v>
+      </c>
+      <c r="G10" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="26" t="inlineStr">
-        <is>
-          <t>BAV99</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">BAV99</t>
         </is>
       </c>
       <c r="B11" s="19" t="inlineStr">
-        <is>
-          <t>Diode Array 1 Pair Series Connection Standard 100V 215mA (DC) Surface Mount TO-236-3, SC-59, SOT-23-3</t>
-        </is>
-      </c>
-      <c r="C11" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Diode Array 1 Pair Series Connection Standard 100V 215mA (DC) Surface Mount TO-236-3, SC-59, SOT-23-3</t>
+        </is>
+      </c>
+      <c r="C11" s="19"/>
       <c r="D11" s="19" t="inlineStr">
-        <is>
-          <t>D4</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">D4</t>
         </is>
       </c>
       <c r="E11" s="19" t="inlineStr">
-        <is>
-          <t>SOT23</t>
-        </is>
-      </c>
-      <c r="F11" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">SOT23</t>
+        </is>
+      </c>
+      <c r="F11" s="27">
+        <v>1</v>
+      </c>
+      <c r="G11" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t>B5819W SL</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">B5819W SL</t>
         </is>
       </c>
       <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>Diode</t>
-        </is>
-      </c>
-      <c r="C12" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Diode</t>
+        </is>
+      </c>
+      <c r="C12" s="19"/>
       <c r="D12" s="19" t="inlineStr">
-        <is>
-          <t>D6, D7, D9</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">D6, D7, D9</t>
         </is>
       </c>
       <c r="E12" s="19" t="inlineStr">
-        <is>
-          <t>SOD-123</t>
-        </is>
-      </c>
-      <c r="F12" s="27" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">SOD-123</t>
+        </is>
+      </c>
+      <c r="F12" s="27">
         <v>3</v>
+      </c>
+      <c r="G12" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="26" t="inlineStr">
-        <is>
-          <t>500mA</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">500mA</t>
         </is>
       </c>
       <c r="B13" s="19" t="inlineStr">
-        <is>
-          <t>Fuse</t>
-        </is>
-      </c>
-      <c r="C13" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Fuse</t>
+        </is>
+      </c>
+      <c r="C13" s="19"/>
       <c r="D13" s="19" t="inlineStr">
-        <is>
-          <t>F1, F2</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">F1, F2</t>
         </is>
       </c>
       <c r="E13" s="19" t="inlineStr">
-        <is>
-          <t>1206</t>
-        </is>
-      </c>
-      <c r="F13" s="27" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">1206</t>
+        </is>
+      </c>
+      <c r="F13" s="27">
         <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="26" t="inlineStr">
-        <is>
-          <t>GZ1608D601TF</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">GZ1608D601TF</t>
         </is>
       </c>
       <c r="B14" s="19" t="inlineStr">
-        <is>
-          <t>Ferrite_Bead</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">Ferrite_Bead</t>
         </is>
       </c>
       <c r="C14" s="19" t="inlineStr">
-        <is>
-          <t>600R@100Mhz</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">600R@100Mhz</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
-        <is>
-          <t>FB1</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">FB1</t>
         </is>
       </c>
       <c r="E14" s="19" t="inlineStr">
-        <is>
-          <t>0603</t>
-        </is>
-      </c>
-      <c r="F14" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">0603</t>
+        </is>
+      </c>
+      <c r="F14" s="27">
+        <v>1</v>
+      </c>
+      <c r="G14" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="26" t="inlineStr">
-        <is>
-          <t>LGS5145</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">LGS5145</t>
         </is>
       </c>
       <c r="B15" s="19" t="inlineStr">
-        <is>
-          <t>60-V, 600-mA High Efficiency Wide Input Voltage Range Buck Converter</t>
-        </is>
-      </c>
-      <c r="C15" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">60-V, 600-mA High Efficiency Wide Input Voltage Range Buck Converter</t>
+        </is>
+      </c>
+      <c r="C15" s="19"/>
       <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>IC1</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">IC1</t>
         </is>
       </c>
       <c r="E15" s="19" t="inlineStr">
-        <is>
-          <t>SOT95P280X110-6N (SOT23-6L)</t>
-        </is>
-      </c>
-      <c r="F15" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">SOT95P280X110-6N (SOT23-6L)</t>
+        </is>
+      </c>
+      <c r="F15" s="27">
+        <v>1</v>
+      </c>
+      <c r="G15" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="26" t="inlineStr">
-        <is>
-          <t>C720477</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">C720477</t>
         </is>
       </c>
       <c r="B16" s="19" t="inlineStr">
-        <is>
-          <t>Tactile Switch</t>
-        </is>
-      </c>
-      <c r="C16" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Tactile Switch</t>
+        </is>
+      </c>
+      <c r="C16" s="19"/>
       <c r="D16" s="19" t="inlineStr">
-        <is>
-          <t>J2, J3</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">J2, J3</t>
         </is>
       </c>
       <c r="E16" s="19" t="inlineStr">
-        <is>
-          <t>TS-1088-AR02016</t>
-        </is>
-      </c>
-      <c r="F16" s="27" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">TS-1088-AR02016</t>
+        </is>
+      </c>
+      <c r="F16" s="27">
         <v>2</v>
+      </c>
+      <c r="G16" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="26" t="inlineStr">
-        <is>
-          <t>C262302</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">C262302</t>
         </is>
       </c>
       <c r="B17" s="19" t="inlineStr">
-        <is>
-          <t>FFC/FPC Connector 10 Position 0.5mm Pitch Single-side Contact/Vertical Surface Mount</t>
-        </is>
-      </c>
-      <c r="C17" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">FFC/FPC Connector 10 Position 0.5mm Pitch Single-side Contact/Vertical Surface Mount</t>
+        </is>
+      </c>
+      <c r="C17" s="19"/>
       <c r="D17" s="19" t="inlineStr">
-        <is>
-          <t>J4</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">J4</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">
-        <is>
-          <t>CONN-TH-10P_AFC11-S10ICC-00</t>
-        </is>
-      </c>
-      <c r="F17" s="27" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">CONN-TH-10P_AFC11-S10ICC-00</t>
+        </is>
+      </c>
+      <c r="F17" s="27">
         <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="26" t="inlineStr">
-        <is>
-          <t>CMI321609X100KT (10uH)</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">CMI321609X100KT (10uH)</t>
         </is>
       </c>
       <c r="B18" s="19" t="inlineStr">
-        <is>
-          <t>15uH</t>
-        </is>
-      </c>
-      <c r="C18" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">15uH</t>
+        </is>
+      </c>
+      <c r="C18" s="19"/>
       <c r="D18" s="19" t="inlineStr">
-        <is>
-          <t>L1</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">L1</t>
         </is>
       </c>
       <c r="E18" s="19" t="inlineStr">
-        <is>
-          <t>L1210</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">L1210</t>
+        </is>
+      </c>
+      <c r="F18" s="27">
+        <v>1</v>
+      </c>
+      <c r="G18" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="26" t="inlineStr">
-        <is>
-          <t>KF2EDGR-3.81-4Pin</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">KF2EDGR-3.81-4Pin</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
-        <is>
-          <t>KF2EDGR-3.81-4Pin</t>
-        </is>
-      </c>
-      <c r="C19" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">KF2EDGR-3.81-4Pin</t>
+        </is>
+      </c>
+      <c r="C19" s="19"/>
       <c r="D19" s="19" t="inlineStr">
-        <is>
-          <t>P5</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">P5</t>
         </is>
       </c>
       <c r="E19" s="19" t="inlineStr">
-        <is>
-          <t>CONN-TH_4P-P3.81_KF2EDGR-3.81-4P</t>
-        </is>
-      </c>
-      <c r="F19" s="27" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">CONN-TH_4P-P3.81_KF2EDGR-3.81-4P</t>
+        </is>
+      </c>
+      <c r="F19" s="27">
         <v>1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="26" t="inlineStr">
-        <is>
-          <t>KF2EDGR-3.5-2Pin</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">KF2EDGR-3.5-2Pin</t>
         </is>
       </c>
       <c r="B20" s="19" t="inlineStr">
-        <is>
-          <t>KF2EDGR-3.5-2Pin</t>
-        </is>
-      </c>
-      <c r="C20" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">KF2EDGR-3.5-2Pin</t>
+        </is>
+      </c>
+      <c r="C20" s="19"/>
       <c r="D20" s="19" t="inlineStr">
-        <is>
-          <t>P6</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">P6</t>
         </is>
       </c>
       <c r="E20" s="19" t="inlineStr">
-        <is>
-          <t>CONN-TH_2P-P3.50_KF2EDGR-3.5</t>
-        </is>
-      </c>
-      <c r="F20" s="27" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">CONN-TH_2P-P3.50_KF2EDGR-3.5</t>
+        </is>
+      </c>
+      <c r="F20" s="27">
         <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="26" t="inlineStr">
-        <is>
-          <t>Header</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">Header</t>
         </is>
       </c>
       <c r="B21" s="19" t="inlineStr">
-        <is>
-          <t>4 Pin male</t>
-        </is>
-      </c>
-      <c r="C21" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">4 Pin male</t>
+        </is>
+      </c>
+      <c r="C21" s="19"/>
       <c r="D21" s="19" t="inlineStr">
-        <is>
-          <t>P7</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">P7</t>
         </is>
       </c>
       <c r="E21" s="19" t="inlineStr">
-        <is>
-          <t>TE_826647-4</t>
-        </is>
-      </c>
-      <c r="F21" s="27" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">TE_826647-4</t>
+        </is>
+      </c>
+      <c r="F21" s="27">
         <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="26" t="inlineStr">
-        <is>
-          <t>AO3400A</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">AO3400A</t>
         </is>
       </c>
       <c r="B22" s="19" t="inlineStr">
-        <is>
-          <t>30V N-Channel MOSFET</t>
-        </is>
-      </c>
-      <c r="C22" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">30V N-Channel MOSFET</t>
+        </is>
+      </c>
+      <c r="C22" s="19"/>
       <c r="D22" s="19" t="inlineStr">
-        <is>
-          <t>Q1</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">Q1</t>
         </is>
       </c>
       <c r="E22" s="19" t="inlineStr">
-        <is>
-          <t>SOT23 Normal</t>
-        </is>
-      </c>
-      <c r="F22" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">SOT23 Normal</t>
+        </is>
+      </c>
+      <c r="F22" s="27">
+        <v>1</v>
+      </c>
+      <c r="G22" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="26" t="inlineStr">
-        <is>
-          <t>AO3401A</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">AO3401A</t>
         </is>
       </c>
       <c r="B23" s="19" t="inlineStr">
-        <is>
-          <t>30V P-Channel MOSFET</t>
-        </is>
-      </c>
-      <c r="C23" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">30V P-Channel MOSFET</t>
+        </is>
+      </c>
+      <c r="C23" s="19"/>
       <c r="D23" s="19" t="inlineStr">
-        <is>
-          <t>Q2</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">Q2</t>
         </is>
       </c>
       <c r="E23" s="19" t="inlineStr">
-        <is>
-          <t>SOT23 Normal</t>
-        </is>
-      </c>
-      <c r="F23" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">SOT23 Normal</t>
+        </is>
+      </c>
+      <c r="F23" s="27">
+        <v>1</v>
+      </c>
+      <c r="G23" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="26" t="inlineStr">
-        <is>
-          <t>MMBT5401</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">MMBT5401</t>
         </is>
       </c>
       <c r="B24" s="19" t="inlineStr">
-        <is>
-          <t>60V, 600 mA, PNP switching transistor</t>
-        </is>
-      </c>
-      <c r="C24" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">60V, 600 mA, PNP switching transistor</t>
+        </is>
+      </c>
+      <c r="C24" s="19"/>
       <c r="D24" s="19" t="inlineStr">
-        <is>
-          <t>Q3</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">Q3</t>
         </is>
       </c>
       <c r="E24" s="19" t="inlineStr">
-        <is>
-          <t>SOT23 Reverse</t>
-        </is>
-      </c>
-      <c r="F24" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">SOT23 Reverse</t>
+        </is>
+      </c>
+      <c r="F24" s="27">
+        <v>1</v>
+      </c>
+      <c r="G24" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="26" t="inlineStr">
-        <is>
-          <t>MMBT5551</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">MMBT5551</t>
         </is>
       </c>
       <c r="B25" s="19" t="inlineStr">
-        <is>
-          <t>NPN General Purpose Transistor</t>
-        </is>
-      </c>
-      <c r="C25" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">NPN General Purpose Transistor</t>
+        </is>
+      </c>
+      <c r="C25" s="19"/>
       <c r="D25" s="19" t="inlineStr">
-        <is>
-          <t>Q5</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">Q5</t>
         </is>
       </c>
       <c r="E25" s="19" t="inlineStr">
-        <is>
-          <t>SOT23 Reverse</t>
-        </is>
-      </c>
-      <c r="F25" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">SOT23 Reverse</t>
+        </is>
+      </c>
+      <c r="F25" s="27">
+        <v>1</v>
+      </c>
+      <c r="G25" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="26" t="inlineStr">
-        <is>
-          <t>100k</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">100k</t>
         </is>
       </c>
       <c r="B26" s="19" t="inlineStr">
-        <is>
-          <t>Resistor</t>
-        </is>
-      </c>
-      <c r="C26" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Resistor</t>
+        </is>
+      </c>
+      <c r="C26" s="19"/>
       <c r="D26" s="19" t="inlineStr">
-        <is>
-          <t>R1, R5, R31</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">R1, R5, R31</t>
         </is>
       </c>
       <c r="E26" s="19" t="inlineStr">
-        <is>
-          <t>R0603</t>
-        </is>
-      </c>
-      <c r="F26" s="27" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">R0603</t>
+        </is>
+      </c>
+      <c r="F26" s="27">
         <v>3</v>
+      </c>
+      <c r="G26" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="26" t="inlineStr">
-        <is>
-          <t>1</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="B27" s="19" t="inlineStr">
-        <is>
-          <t>Resistor</t>
-        </is>
-      </c>
-      <c r="C27" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Resistor</t>
+        </is>
+      </c>
+      <c r="C27" s="19"/>
       <c r="D27" s="19" t="inlineStr">
-        <is>
-          <t>R2</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">R2</t>
         </is>
       </c>
       <c r="E27" s="19" t="inlineStr">
-        <is>
-          <t>R0805</t>
-        </is>
-      </c>
-      <c r="F27" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">R0805</t>
+        </is>
+      </c>
+      <c r="F27" s="27">
+        <v>1</v>
+      </c>
+      <c r="G27" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="26" t="inlineStr">
-        <is>
-          <t>1k</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">1k</t>
         </is>
       </c>
       <c r="B28" s="19" t="inlineStr">
-        <is>
-          <t>Resistor</t>
-        </is>
-      </c>
-      <c r="C28" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Resistor</t>
+        </is>
+      </c>
+      <c r="C28" s="19"/>
       <c r="D28" s="19" t="inlineStr">
-        <is>
-          <t>R3, R29</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">R3, R29</t>
         </is>
       </c>
       <c r="E28" s="19" t="inlineStr">
-        <is>
-          <t>0402</t>
-        </is>
-      </c>
-      <c r="F28" s="27" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">0402</t>
+        </is>
+      </c>
+      <c r="F28" s="27">
         <v>2</v>
+      </c>
+      <c r="G28" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="26" t="inlineStr">
-        <is>
-          <t>100k</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">100k</t>
         </is>
       </c>
       <c r="B29" s="19" t="inlineStr">
-        <is>
-          <t>Resistor</t>
-        </is>
-      </c>
-      <c r="C29" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Resistor</t>
+        </is>
+      </c>
+      <c r="C29" s="19"/>
       <c r="D29" s="19" t="inlineStr">
-        <is>
-          <t>R4</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">R4</t>
         </is>
       </c>
       <c r="E29" s="19" t="inlineStr">
-        <is>
-          <t>0402</t>
-        </is>
-      </c>
-      <c r="F29" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">0402</t>
+        </is>
+      </c>
+      <c r="F29" s="27">
+        <v>1</v>
+      </c>
+      <c r="G29" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="26" t="inlineStr">
-        <is>
-          <t>22k</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">22k</t>
         </is>
       </c>
       <c r="B30" s="19" t="inlineStr">
-        <is>
-          <t>Resistor</t>
-        </is>
-      </c>
-      <c r="C30" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Resistor</t>
+        </is>
+      </c>
+      <c r="C30" s="19"/>
       <c r="D30" s="19" t="inlineStr">
-        <is>
-          <t>R6</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">R6</t>
         </is>
       </c>
       <c r="E30" s="19" t="inlineStr">
-        <is>
-          <t>R1206</t>
-        </is>
-      </c>
-      <c r="F30" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">R1206</t>
+        </is>
+      </c>
+      <c r="F30" s="27">
+        <v>1</v>
+      </c>
+      <c r="G30" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="26" t="inlineStr">
-        <is>
-          <t>10k</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">10k</t>
         </is>
       </c>
       <c r="B31" s="19" t="inlineStr">
-        <is>
-          <t>Resistor</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">Resistor</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
-        <is>
-          <t>1.5k, 1k, 100k, [NoParam]</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">1.5k, 1k, 100k, [NoParam]</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
-        <is>
-          <t>R8, R9, R18, R23, R47</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">R8, R9, R18, R23, R47</t>
         </is>
       </c>
       <c r="E31" s="19" t="inlineStr">
-        <is>
-          <t>0402</t>
-        </is>
-      </c>
-      <c r="F31" s="27" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">0402</t>
+        </is>
+      </c>
+      <c r="F31" s="27">
         <v>5</v>
+      </c>
+      <c r="G31" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="26" t="inlineStr">
-        <is>
-          <t>0</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="B32" s="19" t="inlineStr">
-        <is>
-          <t>Resistor</t>
-        </is>
-      </c>
-      <c r="C32" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Resistor</t>
+        </is>
+      </c>
+      <c r="C32" s="19"/>
       <c r="D32" s="19" t="inlineStr">
-        <is>
-          <t>R10</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">R10</t>
         </is>
       </c>
       <c r="E32" s="19" t="inlineStr">
-        <is>
-          <t>R0603</t>
-        </is>
-      </c>
-      <c r="F32" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">R0603</t>
+        </is>
+      </c>
+      <c r="F32" s="27">
+        <v>1</v>
+      </c>
+      <c r="G32" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="26" t="inlineStr">
-        <is>
-          <t>27</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">27</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
-        <is>
-          <t>0</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
-        <is>
-          <t>100</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">100</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
-        <is>
-          <t>R19, R20</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">R19, R20</t>
         </is>
       </c>
       <c r="E33" s="19" t="inlineStr">
-        <is>
-          <t>0402</t>
-        </is>
-      </c>
-      <c r="F33" s="27" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">0402</t>
+        </is>
+      </c>
+      <c r="F33" s="27">
         <v>2</v>
+      </c>
+      <c r="G33" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="26" t="inlineStr">
-        <is>
-          <t>1.5k</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">1.5k</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
-        <is>
-          <t>Resistor</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">Resistor</t>
         </is>
       </c>
       <c r="C34" s="19" t="inlineStr">
-        <is>
-          <t>1.5k</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">1.5k</t>
         </is>
       </c>
       <c r="D34" s="19" t="inlineStr">
-        <is>
-          <t>R21</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">R21</t>
         </is>
       </c>
       <c r="E34" s="19" t="inlineStr">
-        <is>
-          <t>R0603</t>
-        </is>
-      </c>
-      <c r="F34" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">R0603</t>
+        </is>
+      </c>
+      <c r="F34" s="27">
+        <v>1</v>
+      </c>
+      <c r="G34" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="26" t="inlineStr">
-        <is>
-          <t>10</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="B35" s="19" t="inlineStr">
-        <is>
-          <t>Resistor</t>
-        </is>
-      </c>
-      <c r="C35" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Resistor</t>
+        </is>
+      </c>
+      <c r="C35" s="19"/>
       <c r="D35" s="19" t="inlineStr">
-        <is>
-          <t>R27, R41, R42</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">R27, R41, R42</t>
         </is>
       </c>
       <c r="E35" s="19" t="inlineStr">
-        <is>
-          <t>R0603</t>
-        </is>
-      </c>
-      <c r="F35" s="27" t="n">
+        <v/>
+        <is>
+          <t xml:space="preserve">R0603</t>
+        </is>
+      </c>
+      <c r="F35" s="27">
         <v>3</v>
+      </c>
+      <c r="G35" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="26" t="inlineStr">
-        <is>
-          <t>1M</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">1M</t>
         </is>
       </c>
       <c r="B36" s="19" t="inlineStr">
-        <is>
-          <t>Resistor</t>
-        </is>
-      </c>
-      <c r="C36" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Resistor</t>
+        </is>
+      </c>
+      <c r="C36" s="19"/>
       <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t>R28</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">R28</t>
         </is>
       </c>
       <c r="E36" s="19" t="inlineStr">
-        <is>
-          <t>R0603</t>
-        </is>
-      </c>
-      <c r="F36" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">R0603</t>
+        </is>
+      </c>
+      <c r="F36" s="27">
+        <v>1</v>
+      </c>
+      <c r="G36" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="26" t="inlineStr">
-        <is>
-          <t>4.7k</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">4.7k</t>
         </is>
       </c>
       <c r="B37" s="19" t="inlineStr">
-        <is>
-          <t>Resistor</t>
-        </is>
-      </c>
-      <c r="C37" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Resistor</t>
+        </is>
+      </c>
+      <c r="C37" s="19"/>
       <c r="D37" s="19" t="inlineStr">
-        <is>
-          <t>R30</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">R30</t>
         </is>
       </c>
       <c r="E37" s="19" t="inlineStr">
-        <is>
-          <t>R0603</t>
-        </is>
-      </c>
-      <c r="F37" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">R0603</t>
+        </is>
+      </c>
+      <c r="F37" s="27">
+        <v>1</v>
+      </c>
+      <c r="G37" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="26" t="inlineStr">
-        <is>
-          <t>8.2k</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">8.2k</t>
         </is>
       </c>
       <c r="B38" s="19" t="inlineStr">
-        <is>
-          <t>Resistor</t>
-        </is>
-      </c>
-      <c r="C38" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Resistor</t>
+        </is>
+      </c>
+      <c r="C38" s="19"/>
       <c r="D38" s="19" t="inlineStr">
-        <is>
-          <t>R32</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">R32</t>
         </is>
       </c>
       <c r="E38" s="19" t="inlineStr">
-        <is>
-          <t>R0603</t>
-        </is>
-      </c>
-      <c r="F38" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">R0603</t>
+        </is>
+      </c>
+      <c r="F38" s="27">
+        <v>1</v>
+      </c>
+      <c r="G38" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="26" t="inlineStr">
-        <is>
-          <t>18k</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">18k</t>
         </is>
       </c>
       <c r="B39" s="19" t="inlineStr">
-        <is>
-          <t>Resistor</t>
-        </is>
-      </c>
-      <c r="C39" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Resistor</t>
+        </is>
+      </c>
+      <c r="C39" s="19"/>
       <c r="D39" s="19" t="inlineStr">
-        <is>
-          <t>R33</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">R33</t>
         </is>
       </c>
       <c r="E39" s="19" t="inlineStr">
-        <is>
-          <t>R0603</t>
-        </is>
-      </c>
-      <c r="F39" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">R0603</t>
+        </is>
+      </c>
+      <c r="F39" s="27">
+        <v>1</v>
+      </c>
+      <c r="G39" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="26" t="inlineStr">
-        <is>
-          <t>33k</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">33k</t>
         </is>
       </c>
       <c r="B40" s="19" t="inlineStr">
-        <is>
-          <t>Resistor</t>
-        </is>
-      </c>
-      <c r="C40" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Resistor</t>
+        </is>
+      </c>
+      <c r="C40" s="19"/>
       <c r="D40" s="19" t="inlineStr">
-        <is>
-          <t>R46</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">R46</t>
         </is>
       </c>
       <c r="E40" s="19" t="inlineStr">
-        <is>
-          <t>R0603</t>
-        </is>
-      </c>
-      <c r="F40" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">R0603</t>
+        </is>
+      </c>
+      <c r="F40" s="27">
+        <v>1</v>
+      </c>
+      <c r="G40" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="26" t="inlineStr">
-        <is>
-          <t>CH32V003F4U6</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">CH32V003F4U6</t>
         </is>
       </c>
       <c r="B41" s="19" t="inlineStr">
-        <is>
-          <t>CPU Core:RISC-V CPU Maximum Speed:48MHz Program Storage Size:16KB Number of I/O:18 Applications:-</t>
-        </is>
-      </c>
-      <c r="C41" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">CPU Core:RISC-V CPU Maximum Speed:48MHz Program Storage Size:16KB Number of I/O:18 Applications:-</t>
+        </is>
+      </c>
+      <c r="C41" s="19"/>
       <c r="D41" s="19" t="inlineStr">
-        <is>
-          <t>U1</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">U1</t>
         </is>
       </c>
       <c r="E41" s="19" t="inlineStr">
-        <is>
-          <t>QFN-20_L3.0-W3.0-P0.40-TL-EP1.7</t>
-        </is>
-      </c>
-      <c r="F41" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">QFN-20_L3.0-W3.0-P0.40-TL-EP1.7</t>
+        </is>
+      </c>
+      <c r="F41" s="27">
+        <v>1</v>
+      </c>
+      <c r="G41" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="26" t="inlineStr">
-        <is>
-          <t>LMV331IDBVRG4</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">LMV331IDBVRG4</t>
         </is>
       </c>
       <c r="B42" s="19" t="inlineStr">
-        <is>
-          <t>Single General Purpose Low-Voltage Comparator 5-SOT-23</t>
-        </is>
-      </c>
-      <c r="C42" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">Single General Purpose Low-Voltage Comparator 5-SOT-23</t>
+        </is>
+      </c>
+      <c r="C42" s="19"/>
       <c r="D42" s="19" t="inlineStr">
-        <is>
-          <t>U2</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">U2</t>
         </is>
       </c>
       <c r="E42" s="19" t="inlineStr">
-        <is>
-          <t>SOT23-5</t>
-        </is>
-      </c>
-      <c r="F42" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">SOT23-5</t>
+        </is>
+      </c>
+      <c r="F42" s="27">
+        <v>1</v>
+      </c>
+      <c r="G42" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="26" t="inlineStr">
-        <is>
-          <t>AT24C256C-SSHL-T</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">AT24C256C-SSHL-T</t>
         </is>
       </c>
       <c r="B43" s="19" t="inlineStr">
-        <is>
-          <t>AT24C256C-SSHL-T</t>
-        </is>
-      </c>
-      <c r="C43" s="19" t="n"/>
+        <v/>
+        <is>
+          <t xml:space="preserve">AT24C256C-SSHL-T</t>
+        </is>
+      </c>
+      <c r="C43" s="19"/>
       <c r="D43" s="19" t="inlineStr">
-        <is>
-          <t>U3</t>
+        <v/>
+        <is>
+          <t xml:space="preserve">U3</t>
         </is>
       </c>
       <c r="E43" s="19" t="inlineStr">
-        <is>
-          <t>SOIC127P600X265-8N (SOIC-8)</t>
-        </is>
-      </c>
-      <c r="F43" s="27" t="n">
-        <v>1</v>
+        <v/>
+        <is>
+          <t xml:space="preserve">SOIC127P600X265-8N (SOIC-8)</t>
+        </is>
+      </c>
+      <c r="F43" s="27">
+        <v>1</v>
+      </c>
+      <c r="G43" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>